<commit_message>
Bon de commande : pas de lecteur de badge en plus, celui du nœud salle sert à l'essai réel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/provisoire/docs/Proposition_materiel_CampusTwin.xlsx
+++ b/provisoire/docs/Proposition_materiel_CampusTwin.xlsx
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H90"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" style="11" min="1" max="1"/>
@@ -1521,7 +1521,7 @@
     <row r="34" s="11">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Lecteurs de badge seuls (essai réel dans 2 autres salles)</t>
+          <t>Serveur (une seule machine)</t>
         </is>
       </c>
       <c r="B34" s="5" t="n"/>
@@ -1532,27 +1532,27 @@
       <c r="G34" s="5" t="n"/>
       <c r="H34" s="5" t="n"/>
     </row>
-    <row r="35" s="11">
+    <row r="35" ht="25.5" customHeight="1" s="11">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Carte XIAO ESP32S3 (lecteur de badge)</t>
+          <t>Raspberry Pi 5, 4 Go : seulement si l'IUT n'a pas de Raspberry Pi 3B+/4 ou de vieux PC à nous prêter</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>113991114</t>
+          <t>SC1111</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Seeed Studio</t>
+          <t>Raspberry Pi</t>
         </is>
       </c>
       <c r="D35" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>9</v>
+        <v>95</v>
       </c>
       <c r="F35" s="7">
         <f>D35*E35</f>
@@ -1560,36 +1560,32 @@
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>À commander</t>
-        </is>
-      </c>
-      <c r="H35" s="6" t="inlineStr">
-        <is>
-          <t>lien</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" s="11">
+          <t>Si pas dispo à l'IUT</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="n"/>
+    </row>
+    <row r="36" ht="25.5" customHeight="1" s="11">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Lecteur NFC PN532 V3</t>
+          <t>Accessoires du Raspberry Pi 5 : alimentation 27 W USB-C, carte microSD 64 Go, ventilateur</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>PN532 NFC RFID Module V3</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Elechouse</t>
+          <t>Raspberry Pi</t>
         </is>
       </c>
       <c r="D36" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E36" s="7" t="n">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="F36" s="7">
         <f>D36*E36</f>
@@ -1597,268 +1593,63 @@
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
+          <t>Si pas dispo à l'IUT</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="n"/>
+    </row>
+    <row r="37" s="11"/>
+    <row r="38" s="11">
+      <c r="D38" s="10" t="inlineStr">
+        <is>
           <t>À commander</t>
         </is>
       </c>
-      <c r="H36" s="6" t="n"/>
-    </row>
-    <row r="37" s="11">
-      <c r="A37" s="6" t="inlineStr">
-        <is>
-          <t>LED 5 mm verte et rouge + résistances 220 Ω</t>
-        </is>
-      </c>
-      <c r="B37" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D37" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E37" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F37" s="7">
-        <f>D37*E37</f>
-        <v/>
-      </c>
-      <c r="G37" s="6" t="inlineStr">
-        <is>
-          <t>Stock IUT</t>
-        </is>
-      </c>
-      <c r="H37" s="6" t="n"/>
-    </row>
-    <row r="38" s="11">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>Buzzer actif 3,3 V</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D38" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E38" s="7" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="F38" s="7">
-        <f>D38*E38</f>
-        <v/>
-      </c>
-      <c r="G38" s="6" t="inlineStr">
-        <is>
-          <t>Stock IUT</t>
-        </is>
-      </c>
-      <c r="H38" s="6" t="n"/>
+      <c r="F38" s="9">
+        <f>SUMIF(G6:G36,"À commander",F6:F36)</f>
+        <v/>
+      </c>
     </row>
     <row r="39" s="11">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>Boîtier plastique pour le lecteur</t>
-        </is>
-      </c>
-      <c r="B39" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C39" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D39" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E39" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="F39" s="7">
-        <f>D39*E39</f>
-        <v/>
-      </c>
-      <c r="G39" s="6" t="inlineStr">
-        <is>
-          <t>Stock IUT</t>
-        </is>
-      </c>
-      <c r="H39" s="6" t="n"/>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>Stock IUT (si à acheter)</t>
+        </is>
+      </c>
+      <c r="F39" s="9">
+        <f>SUMIF(G6:G36,"Stock IUT",F6:F36)</f>
+        <v/>
+      </c>
     </row>
     <row r="40" s="11">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>Alimentation USB-C 5 V, 1 A</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C40" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D40" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E40" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="F40" s="7">
-        <f>D40*E40</f>
-        <v/>
-      </c>
-      <c r="G40" s="6" t="inlineStr">
-        <is>
-          <t>À commander</t>
-        </is>
-      </c>
-      <c r="H40" s="6" t="n"/>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>Si pas dispo à l'IUT</t>
+        </is>
+      </c>
+      <c r="F40" s="9">
+        <f>SUMIF(G6:G36,"Si pas dispo à l'IUT",F6:F36)</f>
+        <v/>
+      </c>
     </row>
     <row r="41" s="11">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>Serveur (une seule machine)</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="n"/>
-      <c r="C41" s="5" t="n"/>
-      <c r="D41" s="5" t="n"/>
-      <c r="E41" s="5" t="n"/>
-      <c r="F41" s="5" t="n"/>
-      <c r="G41" s="5" t="n"/>
-      <c r="H41" s="5" t="n"/>
-    </row>
-    <row r="42" ht="25.5" customHeight="1" s="11">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>Raspberry Pi 5, 4 Go : seulement si l'IUT n'a pas de Raspberry Pi 3B+/4 ou de vieux PC à nous prêter</t>
-        </is>
-      </c>
-      <c r="B42" s="6" t="inlineStr">
-        <is>
-          <t>SC1111</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="inlineStr">
-        <is>
-          <t>Raspberry Pi</t>
-        </is>
-      </c>
-      <c r="D42" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E42" s="7" t="n">
-        <v>95</v>
-      </c>
-      <c r="F42" s="7">
-        <f>D42*E42</f>
-        <v/>
-      </c>
-      <c r="G42" s="6" t="inlineStr">
-        <is>
-          <t>Si pas dispo à l'IUT</t>
-        </is>
-      </c>
-      <c r="H42" s="6" t="n"/>
-    </row>
-    <row r="43" ht="25.5" customHeight="1" s="11">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>Accessoires du Raspberry Pi 5 : alimentation 27 W USB-C, carte microSD 64 Go, ventilateur</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C43" s="6" t="inlineStr">
-        <is>
-          <t>Raspberry Pi</t>
-        </is>
-      </c>
-      <c r="D43" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E43" s="7" t="n">
-        <v>33</v>
-      </c>
-      <c r="F43" s="7">
-        <f>D43*E43</f>
-        <v/>
-      </c>
-      <c r="G43" s="6" t="inlineStr">
-        <is>
-          <t>Si pas dispo à l'IUT</t>
-        </is>
-      </c>
-      <c r="H43" s="6" t="n"/>
-    </row>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>Option</t>
+        </is>
+      </c>
+      <c r="F41" s="9">
+        <f>SUMIF(G6:G36,"Option",F6:F36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" s="11"/>
+    <row r="43" s="11"/>
     <row r="44" s="11"/>
-    <row r="45" s="11">
-      <c r="D45" s="10" t="inlineStr">
-        <is>
-          <t>À commander</t>
-        </is>
-      </c>
-      <c r="F45" s="9">
-        <f>SUMIF(G6:G43,"À commander",F6:F43)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" s="11">
-      <c r="D46" s="10" t="inlineStr">
-        <is>
-          <t>Stock IUT (si à acheter)</t>
-        </is>
-      </c>
-      <c r="F46" s="9">
-        <f>SUMIF(G6:G43,"Stock IUT",F6:F43)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" s="11">
-      <c r="D47" s="10" t="inlineStr">
-        <is>
-          <t>Si pas dispo à l'IUT</t>
-        </is>
-      </c>
-      <c r="F47" s="9">
-        <f>SUMIF(G6:G43,"Si pas dispo à l'IUT",F6:F43)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" s="11">
-      <c r="D48" s="10" t="inlineStr">
-        <is>
-          <t>Option</t>
-        </is>
-      </c>
-      <c r="F48" s="9">
-        <f>SUMIF(G6:G43,"Option",F6:F43)</f>
-        <v/>
-      </c>
-    </row>
+    <row r="45" s="11"/>
+    <row r="46" s="11"/>
+    <row r="47" s="11"/>
+    <row r="48" s="11"/>
     <row r="49" s="11"/>
     <row r="50" s="11"/>
     <row r="51" s="11"/>
@@ -1870,15 +1661,36 @@
     <row r="57" s="11"/>
     <row r="58" s="11"/>
     <row r="59" s="11"/>
+    <row r="60" s="11"/>
+    <row r="61" s="11"/>
+    <row r="62" s="11"/>
+    <row r="63" s="11"/>
+    <row r="64" s="11"/>
+    <row r="65" s="11"/>
+    <row r="66" s="11"/>
+    <row r="67" s="11"/>
+    <row r="68" s="11"/>
+    <row r="69" s="11"/>
+    <row r="70" s="11"/>
+    <row r="71" s="11"/>
+    <row r="72" s="11"/>
+    <row r="73" s="11"/>
+    <row r="74" s="11"/>
+    <row r="75" s="11"/>
+    <row r="76" s="11"/>
+    <row r="77" s="11"/>
+    <row r="78" s="11"/>
+    <row r="79" s="11"/>
+    <row r="90"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D39:E39"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="G6:G43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"À commander,Stock IUT,Si pas dispo à l'IUT,Option,Alternative,Déjà dispo"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1893,7 +1705,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Compter avec les ondes Wi-Fi : deux cartes ESP32-S3 et le CSI
- firmware/ondes_wifi : l'émetteur envoie 50 paquets ESP-NOW par seconde, le récepteur lit le
  CSI des 52 sous-porteuses et envoie toutes les 10 s le mouvement mesuré (compile pour les deux rôles).
- serveur/ondes.py : niveau de la salle vide appris, présence, mesures gardées avec le comptage de la
  porte dans serveur/ondes.csv pour apprendre à compter.
- outils/ondes_wifi.py : la présence et le comptage par les ondes comparés à la porte.
- Simulation (relation inventée), fiche de séance, test_ondes.py, 2 XIAO de plus dans la commande.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/provisoire/docs/Proposition_materiel_CampusTwin.xlsx
+++ b/provisoire/docs/Proposition_materiel_CampusTwin.xlsx
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H90"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" style="11" min="1" max="1"/>
@@ -1447,7 +1447,7 @@
     <row r="32" s="11">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Carte XIAO ESP32S3 (essai de détection par Wi-Fi)</t>
+          <t>Carte XIAO ESP32S3 (mesure des ondes Wi-Fi : émetteur et récepteur)</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>Option</t>
+          <t>À commander</t>
         </is>
       </c>
       <c r="H32" s="8" t="inlineStr">
@@ -1681,7 +1681,6 @@
     <row r="77" s="11"/>
     <row r="78" s="11"/>
     <row r="79" s="11"/>
-    <row r="90"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="D38:E38"/>

</xml_diff>